<commit_message>
LØM-app 2.6.5: forkortelser skrevet ut og formler med ord i alle kapitler
</commit_message>
<xml_diff>
--- a/pensum/ma02/MA02_Klasseoppgaver_v5.xlsx
+++ b/pensum/ma02/MA02_Klasseoppgaver_v5.xlsx
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Kort oppsummert: Forbrukeren går gjennom fem trinn: behov, søk etter alternativer, vurdering av alternativer, kjøp og evaluering. Et behov er en følt mangeltilstand som søkes fjernet; Maslow ordner behovene i fem nivåer. Ved større kjøp har familien fire kjøpsroller: påvirker, bruker, beslutningstager og kjøper. Etter kjøpet kommer ofte etterkjøpskvalene, og selgeren kan dempe dem ved å være tilgjengelig.</t>
   </si>
   <si>
-    <t xml:space="preserve">Familien Lunde bor i en enebolig i Oslo og har bestilt elbil med levering i mars. De har fått tre tilbud på ladeboks: Nordlys 19 900 kr, tilbud B 17 500 kr og tilbud C 18 900 kr, alle inkl. mva og montering. Datteren på 17 har funnet et bestemt merke og mast om det i ukevis. Naboen har ladeboks fra Nordlys og anbefalte dem. Far sier at han først og fremst vil slippe å dra skjøteledning ut av kjellervinduet hele vinteren. Mor og far bestemmer sammen; far ringer, bestiller og betaler. Nordlys fikk jobben. To uker etter montering sier mor: «Burde vi ikke tatt den billigste?» Bruk læreboka kap. 2.2–2.3 og svar på deloppgavene.</t>
+    <t xml:space="preserve">Familien Lunde bor i en enebolig i Oslo og har bestilt elbil med levering i mars. De har fått tre tilbud på ladeboks: Nordlys 19 900 kr, tilbud B 17 500 kr og tilbud C 18 900 kr, alle inkludert merverdiavgift og montering. Datteren på 17 har funnet et bestemt merke og mast om det i ukevis. Naboen har ladeboks fra Nordlys og anbefalte dem. Far sier at han først og fremst vil slippe å dra skjøteledning ut av kjellervinduet hele vinteren. Mor og far bestemmer sammen; far ringer, bestiller og betaler. Nordlys fikk jobben. To uker etter montering sier mor: «Burde vi ikke tatt den billigste?» Bruk læreboka kap. 2.2–2.3 og svar på deloppgavene.</t>
   </si>
   <si>
     <t xml:space="preserve">Forutsetning</t>
@@ -323,7 +323,7 @@
     <t xml:space="preserve">Kort oppsummert: Et borettslag kjøper som en bedrift: formalisert, etter regler som skal sikre riktig vare, mengde, pris og tidspunkt og redusere kjøpsrisikoen. En nyanskaffelse går gjennom alle åtte trinnene i tabell 2.1, og leverandøren velges etter tekniske, økonomiske og tidsplanmessige krav. Kjøpsrollene er initiativtager, påvirker, bruker, beslutningstager, godkjenner, innkjøper og portvakt.</t>
   </si>
   <si>
-    <t xml:space="preserve">Borettslaget har 48 leiligheter og 52 parkeringsplasser og har aldri hatt ladeanlegg. Styrelederen tok initiativet etter klager fra beboere. En beboer som er elektroingeniør, er den eneste i styret som forstår lastbalansering, og styret stoler på ham. En innleid rådgiver skrev kravspesifikasjonen. Forretningsføreren sorterer henvendelsene fra leverandører og sender ut forespørslene. Styret på fem innstiller på leverandør, og generalforsamlingen i mai vedtar låneopptaket. Anlegget koster 1 350 000 kr inkl. mva. Laget er ikke mva-registrert, så hele summen må lånes. Nordlys leverte det billigste av tre anbud og tapte. Ida sendte dette til styret: «Hei! Vedlagt følger vårt tilbud, 1 350 000 kr inkl. mva. Vi bruker markedets beste lader med dynamisk lastbalansering. Prisen er den laveste du får i byen. Ring meg gjerne direkte hvis du lurer på noe teknisk. Vi kan starte om tre uker.»</t>
+    <t xml:space="preserve">Borettslaget har 48 leiligheter og 52 parkeringsplasser og har aldri hatt ladeanlegg. Styrelederen tok initiativet etter klager fra beboere. En beboer som er elektroingeniør, er den eneste i styret som forstår lastbalansering, og styret stoler på ham. En innleid rådgiver skrev kravspesifikasjonen. Forretningsføreren sorterer henvendelsene fra leverandører og sender ut forespørslene. Styret på fem innstiller på leverandør, og generalforsamlingen i mai vedtar låneopptaket. Anlegget koster 1 350 000 kr inkludert merverdiavgift (mva). Laget er ikke mva-registrert, så hele summen må lånes. Nordlys leverte det billigste av tre anbud og tapte. Ida sendte dette til styret: «Hei! Vedlagt følger vårt tilbud, 1 350 000 kr inkludert mva. Vi bruker markedets beste lader med dynamisk lastbalansering. Prisen er den laveste du får i byen. Ring meg gjerne direkte hvis du lurer på noe teknisk. Vi kan starte om tre uker.»</t>
   </si>
   <si>
     <t xml:space="preserve">Borettslaget</t>
@@ -335,13 +335,13 @@
     <t xml:space="preserve">Anlegget</t>
   </si>
   <si>
-    <t xml:space="preserve">Lading på alle plasser, 1 350 000 kr inkl. mva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laget er ikke mva-registrert: alt lånes</t>
+    <t xml:space="preserve">Lading på alle plasser, 1 350 000 kr inkludert merverdiavgift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merverdiavgift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laget er ikke registrert for merverdiavgift: alt lånes</t>
   </si>
   <si>
     <t xml:space="preserve">Styrelederen</t>
@@ -380,10 +380,10 @@
     <t xml:space="preserve">Billigst av tre anbud, men tapte</t>
   </si>
   <si>
-    <t xml:space="preserve">a)  Hva koster anlegget per leilighet, i kroner? Laget er ikke mva-registrert, så bruk prisen inkl. mva og del på antall leiligheter.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pris per enhet = totalpris / antall enheter. Pris uten mva = pris inkl. mva / 1,25 (mva 25 %, merverdiavgiftsloven § 5-1). Regnestykket står ikke i Markedsføring kap. 2, men det handler om «riktig pris», ett av de fire kravene i 2.4.</t>
+    <t xml:space="preserve">a)  Hva koster anlegget per leilighet, i kroner? Laget er ikke registrert for merverdiavgift, så bruk prisen inkludert merverdiavgift og del på antall leiligheter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pris per enhet = totalpris / antall enheter. Pris uten merverdiavgift = pris med merverdiavgift / 1,25 (merverdiavgift 25 %, merverdiavgiftsloven § 5-1). Regnestykket står ikke i Markedsføring kap. 2, men det handler om «riktig pris», ett av de fire kravene i 2.4.</t>
   </si>
   <si>
     <t xml:space="preserve">b)  Borettslaget har aldri hatt ladeanlegg. Hvilken kjøpssituasjon er det?   A: Nyanskaffelse   B: Overveid gjenkjøp   C: Rent gjenkjøp   (skriv bokstaven)</t>
@@ -419,7 +419,7 @@
     <t xml:space="preserve">Pris og situasjon</t>
   </si>
   <si>
-    <t xml:space="preserve">Laget får ikke fradrag for mva, så del hele 1 350 000 på 48. Har borettslaget kjøpt et slikt anlegg før? Da vet du situasjonen.</t>
+    <t xml:space="preserve">Laget får ikke fradrag for merverdiavgift, så del hele 1 350 000 på 48. Har borettslaget kjøpt et slikt anlegg før? Da vet du situasjonen.</t>
   </si>
   <si>
     <t xml:space="preserve">Rollene og valget</t>

</xml_diff>